<commit_message>
Added prints to model selector
</commit_message>
<xml_diff>
--- a/runtimesheet.xlsx
+++ b/runtimesheet.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,43 +500,43 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>250163</v>
+        <v>252233</v>
       </c>
       <c r="C2" t="n">
-        <v>250163.2</v>
+        <v>252233.4</v>
       </c>
       <c r="D2" t="n">
-        <v>219.4</v>
+        <v>365.9</v>
       </c>
       <c r="E2" t="n">
-        <v>147059</v>
+        <v>172413.3</v>
       </c>
       <c r="F2" t="n">
-        <v>2.6</v>
+        <v>1.5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="H2" t="n">
-        <v>12.9</v>
+        <v>8.5</v>
       </c>
       <c r="I2" t="n">
-        <v>183.8</v>
+        <v>328.7</v>
       </c>
       <c r="J2" t="n">
-        <v>2.8</v>
+        <v>3.7</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="M2" t="n">
-        <v>16.4</v>
+        <v>17.3</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
@@ -544,40 +544,40 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>250163.2</v>
+        <v>252233.4</v>
       </c>
       <c r="C3" t="n">
-        <v>250163.3</v>
+        <v>252233.5</v>
       </c>
       <c r="D3" t="n">
-        <v>122.5</v>
+        <v>154.1</v>
       </c>
       <c r="E3" t="n">
-        <v>9.1</v>
+        <v>5.5</v>
       </c>
       <c r="F3" t="n">
-        <v>1.5</v>
+        <v>3.4</v>
       </c>
       <c r="G3" t="n">
         <v>2.7</v>
       </c>
       <c r="H3" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>100.8</v>
+        <v>135.2</v>
       </c>
       <c r="J3" t="n">
-        <v>6.2</v>
+        <v>2.1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="L3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M3" t="n">
         <v>0.3</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.5</v>
       </c>
       <c r="N3" t="n">
         <v>0.1</v>
@@ -588,31 +588,31 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>250163.3</v>
+        <v>252233.5</v>
       </c>
       <c r="C4" t="n">
-        <v>250163.4</v>
+        <v>252233.7</v>
       </c>
       <c r="D4" t="n">
-        <v>81.59999999999999</v>
+        <v>142.3</v>
       </c>
       <c r="E4" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="F4" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G4" t="n">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="I4" t="n">
-        <v>64.59999999999999</v>
+        <v>126.9</v>
       </c>
       <c r="J4" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="K4" t="n">
         <v>0.5</v>
@@ -621,7 +621,7 @@
         <v>0.2</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="N4" t="n">
         <v>0.1</v>
@@ -632,28 +632,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>250163.4</v>
+        <v>252233.7</v>
       </c>
       <c r="C5" t="n">
-        <v>250163.5</v>
+        <v>252233.8</v>
       </c>
       <c r="D5" t="n">
-        <v>78.59999999999999</v>
+        <v>140.8</v>
       </c>
       <c r="E5" t="n">
-        <v>9.4</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="G5" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="H5" t="n">
-        <v>8.1</v>
+        <v>8.4</v>
       </c>
       <c r="I5" t="n">
-        <v>64.5</v>
+        <v>126.2</v>
       </c>
       <c r="J5" t="n">
         <v>2.1</v>
@@ -662,13 +662,13 @@
         <v>0.4</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M5" t="n">
         <v>0.3</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6">
@@ -676,43 +676,43 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>250163.5</v>
+        <v>252233.8</v>
       </c>
       <c r="C6" t="n">
-        <v>250163.6</v>
+        <v>252233.9</v>
       </c>
       <c r="D6" t="n">
-        <v>79.09999999999999</v>
+        <v>141.1</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>6.2</v>
       </c>
       <c r="F6" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="G6" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="H6" t="n">
-        <v>7.5</v>
+        <v>8.4</v>
       </c>
       <c r="I6" t="n">
-        <v>60.7</v>
+        <v>125.8</v>
       </c>
       <c r="J6" t="n">
-        <v>7.6</v>
+        <v>2.3</v>
       </c>
       <c r="K6" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -720,43 +720,43 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>250163.6</v>
+        <v>252233.9</v>
       </c>
       <c r="C7" t="n">
-        <v>250163.7</v>
+        <v>252234.1</v>
       </c>
       <c r="D7" t="n">
-        <v>73.2</v>
+        <v>140.8</v>
       </c>
       <c r="E7" t="n">
-        <v>10.3</v>
+        <v>6.4</v>
       </c>
       <c r="F7" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="H7" t="n">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>60.3</v>
+        <v>126.1</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="K7" t="n">
         <v>0.4</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M7" t="n">
         <v>0.3</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8">
@@ -764,43 +764,43 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>250163.7</v>
+        <v>252234.1</v>
       </c>
       <c r="C8" t="n">
-        <v>250163.7</v>
+        <v>252234.2</v>
       </c>
       <c r="D8" t="n">
-        <v>73.40000000000001</v>
+        <v>141.6</v>
       </c>
       <c r="E8" t="n">
-        <v>10.7</v>
+        <v>6.5</v>
       </c>
       <c r="F8" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G8" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="H8" t="n">
-        <v>7.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>60.8</v>
+        <v>127.1</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="K8" t="n">
         <v>0.4</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9">
@@ -808,43 +808,43 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>250163.7</v>
+        <v>252234.2</v>
       </c>
       <c r="C9" t="n">
-        <v>250163.8</v>
+        <v>252234.4</v>
       </c>
       <c r="D9" t="n">
-        <v>76.5</v>
+        <v>138.7</v>
       </c>
       <c r="E9" t="n">
-        <v>11</v>
+        <v>6.5</v>
       </c>
       <c r="F9" t="n">
-        <v>1.2</v>
+        <v>2.3</v>
       </c>
       <c r="G9" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="H9" t="n">
-        <v>6.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>63.9</v>
+        <v>122.8</v>
       </c>
       <c r="J9" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="K9" t="n">
         <v>0.4</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M9" t="n">
         <v>0.3</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
@@ -852,28 +852,28 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>250163.8</v>
+        <v>252234.4</v>
       </c>
       <c r="C10" t="n">
-        <v>250163.9</v>
+        <v>252234.5</v>
       </c>
       <c r="D10" t="n">
-        <v>74.8</v>
+        <v>136.1</v>
       </c>
       <c r="E10" t="n">
-        <v>11.2</v>
+        <v>6.6</v>
       </c>
       <c r="F10" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="H10" t="n">
-        <v>7.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>62.4</v>
+        <v>120.6</v>
       </c>
       <c r="J10" t="n">
         <v>2.1</v>
@@ -882,13 +882,13 @@
         <v>0.4</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M10" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
@@ -896,34 +896,34 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>250163.9</v>
+        <v>252234.5</v>
       </c>
       <c r="C11" t="n">
-        <v>250164</v>
+        <v>252234.6</v>
       </c>
       <c r="D11" t="n">
-        <v>80.90000000000001</v>
+        <v>133.9</v>
       </c>
       <c r="E11" t="n">
-        <v>11.4</v>
+        <v>6.7</v>
       </c>
       <c r="F11" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="G11" t="n">
         <v>1.2</v>
       </c>
       <c r="H11" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
       <c r="I11" t="n">
-        <v>67.59999999999999</v>
+        <v>119.8</v>
       </c>
       <c r="J11" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
       <c r="K11" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L11" t="n">
         <v>0.2</v>
@@ -940,34 +940,34 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>250164</v>
+        <v>252234.6</v>
       </c>
       <c r="C12" t="n">
-        <v>250164</v>
+        <v>252234.8</v>
       </c>
       <c r="D12" t="n">
-        <v>82</v>
+        <v>137.3</v>
       </c>
       <c r="E12" t="n">
-        <v>11.5</v>
+        <v>6.7</v>
       </c>
       <c r="F12" t="n">
-        <v>2.3</v>
+        <v>1.5</v>
       </c>
       <c r="G12" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="H12" t="n">
-        <v>8.4</v>
+        <v>8.1</v>
       </c>
       <c r="I12" t="n">
-        <v>66.7</v>
+        <v>123.7</v>
       </c>
       <c r="J12" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="K12" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L12" t="n">
         <v>0.2</v>
@@ -984,43 +984,43 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>250164</v>
+        <v>252234.8</v>
       </c>
       <c r="C13" t="n">
-        <v>250164.1</v>
+        <v>252234.9</v>
       </c>
       <c r="D13" t="n">
-        <v>77</v>
+        <v>138.7</v>
       </c>
       <c r="E13" t="n">
-        <v>12.2</v>
+        <v>7.1</v>
       </c>
       <c r="F13" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>63.7</v>
+        <v>124.5</v>
       </c>
       <c r="J13" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K13" t="n">
         <v>0.4</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M13" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="N13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="14">
@@ -1028,34 +1028,34 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>250164.1</v>
+        <v>252234.9</v>
       </c>
       <c r="C14" t="n">
-        <v>250164.2</v>
+        <v>252235</v>
       </c>
       <c r="D14" t="n">
-        <v>75.59999999999999</v>
+        <v>137.9</v>
       </c>
       <c r="E14" t="n">
-        <v>12.9</v>
+        <v>7.2</v>
       </c>
       <c r="F14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G14" t="n">
         <v>1.1</v>
       </c>
-      <c r="G14" t="n">
-        <v>1.2</v>
-      </c>
       <c r="H14" t="n">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="I14" t="n">
-        <v>61</v>
+        <v>124.2</v>
       </c>
       <c r="J14" t="n">
-        <v>3.4</v>
+        <v>2</v>
       </c>
       <c r="K14" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L14" t="n">
         <v>0.2</v>
@@ -1072,43 +1072,43 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>250164.2</v>
+        <v>252235</v>
       </c>
       <c r="C15" t="n">
-        <v>250164.3</v>
+        <v>252235.2</v>
       </c>
       <c r="D15" t="n">
-        <v>73.90000000000001</v>
+        <v>138.5</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>7.2</v>
       </c>
       <c r="F15" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="H15" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I15" t="n">
-        <v>61</v>
+        <v>124.4</v>
       </c>
       <c r="J15" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K15" t="n">
         <v>0.4</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M15" t="n">
         <v>0.3</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16">
@@ -1116,34 +1116,34 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>250164.3</v>
+        <v>252235.2</v>
       </c>
       <c r="C16" t="n">
-        <v>250164.3</v>
+        <v>252235.3</v>
       </c>
       <c r="D16" t="n">
-        <v>71.7</v>
+        <v>143.5</v>
       </c>
       <c r="E16" t="n">
-        <v>13</v>
+        <v>7.2</v>
       </c>
       <c r="F16" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="G16" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H16" t="n">
-        <v>6.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>60.5</v>
+        <v>127.8</v>
       </c>
       <c r="J16" t="n">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L16" t="n">
         <v>0.2</v>
@@ -1152,7 +1152,7 @@
         <v>0.4</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="17">
@@ -1160,34 +1160,34 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>250164.3</v>
+        <v>252235.3</v>
       </c>
       <c r="C17" t="n">
-        <v>250164.4</v>
+        <v>252235.5</v>
       </c>
       <c r="D17" t="n">
-        <v>77.59999999999999</v>
+        <v>156.4</v>
       </c>
       <c r="E17" t="n">
-        <v>13.2</v>
+        <v>7.2</v>
       </c>
       <c r="F17" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="G17" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="H17" t="n">
-        <v>7.9</v>
+        <v>10.4</v>
       </c>
       <c r="I17" t="n">
-        <v>64.2</v>
+        <v>138.4</v>
       </c>
       <c r="J17" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="K17" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L17" t="n">
         <v>0.2</v>
@@ -1204,28 +1204,28 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>250164.4</v>
+        <v>252235.5</v>
       </c>
       <c r="C18" t="n">
-        <v>250164.5</v>
+        <v>252235.6</v>
       </c>
       <c r="D18" t="n">
-        <v>73.7</v>
+        <v>138</v>
       </c>
       <c r="E18" t="n">
-        <v>13.1</v>
+        <v>7.1</v>
       </c>
       <c r="F18" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="G18" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H18" t="n">
-        <v>7.9</v>
+        <v>9.5</v>
       </c>
       <c r="I18" t="n">
-        <v>60.2</v>
+        <v>122.2</v>
       </c>
       <c r="J18" t="n">
         <v>2.1</v>
@@ -1237,7 +1237,7 @@
         <v>0.2</v>
       </c>
       <c r="M18" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N18" t="n">
         <v>0.1</v>
@@ -1248,31 +1248,31 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>250164.5</v>
+        <v>252235.6</v>
       </c>
       <c r="C19" t="n">
-        <v>250164.6</v>
+        <v>252235.8</v>
       </c>
       <c r="D19" t="n">
-        <v>75.2</v>
+        <v>138.7</v>
       </c>
       <c r="E19" t="n">
-        <v>13.1</v>
+        <v>7.1</v>
       </c>
       <c r="F19" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="G19" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="I19" t="n">
-        <v>61.8</v>
+        <v>124.4</v>
       </c>
       <c r="J19" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="K19" t="n">
         <v>0.4</v>
@@ -1292,31 +1292,31 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>250164.6</v>
+        <v>252235.8</v>
       </c>
       <c r="C20" t="n">
-        <v>250164.6</v>
+        <v>252235.9</v>
       </c>
       <c r="D20" t="n">
-        <v>72.8</v>
+        <v>136.6</v>
       </c>
       <c r="E20" t="n">
-        <v>13.1</v>
+        <v>7.1</v>
       </c>
       <c r="F20" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="G20" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H20" t="n">
-        <v>7.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>59.6</v>
+        <v>122.2</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="K20" t="n">
         <v>0.4</v>
@@ -1328,7 +1328,7 @@
         <v>0.3</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="21">
@@ -1336,40 +1336,40 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>250164.6</v>
+        <v>252235.9</v>
       </c>
       <c r="C21" t="n">
-        <v>250164.7</v>
+        <v>252236</v>
       </c>
       <c r="D21" t="n">
-        <v>76.09999999999999</v>
+        <v>139.9</v>
       </c>
       <c r="E21" t="n">
-        <v>13.1</v>
+        <v>7.1</v>
       </c>
       <c r="F21" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G21" t="n">
         <v>1.2</v>
       </c>
       <c r="H21" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I21" t="n">
-        <v>62.7</v>
+        <v>125.7</v>
       </c>
       <c r="J21" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="K21" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="M21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N21" t="n">
         <v>0.1</v>
@@ -1380,40 +1380,40 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>250164.7</v>
+        <v>252236</v>
       </c>
       <c r="C22" t="n">
-        <v>250164.8</v>
+        <v>252236.2</v>
       </c>
       <c r="D22" t="n">
-        <v>77.3</v>
+        <v>139.2</v>
       </c>
       <c r="E22" t="n">
-        <v>13.2</v>
+        <v>7.1</v>
       </c>
       <c r="F22" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="G22" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="H22" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="I22" t="n">
-        <v>63.1</v>
+        <v>124.6</v>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="K22" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L22" t="n">
         <v>0.2</v>
       </c>
       <c r="M22" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N22" t="n">
         <v>0.1</v>
@@ -1424,31 +1424,31 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>250164.8</v>
+        <v>252236.2</v>
       </c>
       <c r="C23" t="n">
-        <v>250164.9</v>
+        <v>252236.3</v>
       </c>
       <c r="D23" t="n">
-        <v>79</v>
+        <v>139.3</v>
       </c>
       <c r="E23" t="n">
-        <v>13.3</v>
+        <v>7.1</v>
       </c>
       <c r="F23" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="G23" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="H23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I23" t="n">
-        <v>64.8</v>
+        <v>124.2</v>
       </c>
       <c r="J23" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="K23" t="n">
         <v>0.4</v>
@@ -1457,7 +1457,7 @@
         <v>0.2</v>
       </c>
       <c r="M23" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N23" t="n">
         <v>0.1</v>
@@ -1468,31 +1468,31 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>250164.9</v>
+        <v>252236.3</v>
       </c>
       <c r="C24" t="n">
-        <v>250165</v>
+        <v>252236.5</v>
       </c>
       <c r="D24" t="n">
-        <v>75.40000000000001</v>
+        <v>140.8</v>
       </c>
       <c r="E24" t="n">
-        <v>13.3</v>
+        <v>7.1</v>
       </c>
       <c r="F24" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="G24" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="H24" t="n">
-        <v>7.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I24" t="n">
-        <v>62.3</v>
+        <v>125.2</v>
       </c>
       <c r="J24" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="K24" t="n">
         <v>0.4</v>
@@ -1504,7 +1504,7 @@
         <v>0.4</v>
       </c>
       <c r="N24" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25">
@@ -1512,31 +1512,31 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>250165</v>
+        <v>252236.5</v>
       </c>
       <c r="C25" t="n">
-        <v>250165</v>
+        <v>252236.6</v>
       </c>
       <c r="D25" t="n">
-        <v>77.2</v>
+        <v>138.5</v>
       </c>
       <c r="E25" t="n">
-        <v>13.3</v>
+        <v>7.1</v>
       </c>
       <c r="F25" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="G25" t="n">
         <v>0.9</v>
       </c>
       <c r="H25" t="n">
-        <v>7.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I25" t="n">
-        <v>64.8</v>
+        <v>124.1</v>
       </c>
       <c r="J25" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K25" t="n">
         <v>0.4</v>
@@ -1545,10 +1545,10 @@
         <v>0.2</v>
       </c>
       <c r="M25" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26">
@@ -1556,32 +1556,32 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>250165</v>
+        <v>252236.6</v>
       </c>
       <c r="C26" t="n">
-        <v>250165.1</v>
+        <v>252236.7</v>
       </c>
       <c r="D26" t="n">
-        <v>76</v>
+        <v>136.4</v>
       </c>
       <c r="E26" t="n">
-        <v>13.2</v>
+        <v>7.1</v>
       </c>
       <c r="F26" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H26" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="I26" t="n">
+        <v>123</v>
+      </c>
+      <c r="J26" t="n">
         <v>2.1</v>
       </c>
-      <c r="G26" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="H26" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="I26" t="n">
-        <v>62</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1.9</v>
-      </c>
       <c r="K26" t="n">
         <v>0.4</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>0.2</v>
       </c>
       <c r="M26" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N26" t="n">
         <v>0.1</v>
@@ -1600,43 +1600,43 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>250165.1</v>
+        <v>252236.7</v>
       </c>
       <c r="C27" t="n">
-        <v>250165.2</v>
+        <v>252236.9</v>
       </c>
       <c r="D27" t="n">
-        <v>71.8</v>
+        <v>135.5</v>
       </c>
       <c r="E27" t="n">
-        <v>13.2</v>
+        <v>7.1</v>
       </c>
       <c r="F27" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G27" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
         <v>8.1</v>
       </c>
       <c r="I27" t="n">
-        <v>58.4</v>
+        <v>121.8</v>
       </c>
       <c r="J27" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K27" t="n">
         <v>0.4</v>
       </c>
       <c r="L27" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M27" t="n">
         <v>0.3</v>
       </c>
       <c r="N27" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28">
@@ -1644,31 +1644,31 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>250165.2</v>
+        <v>252236.9</v>
       </c>
       <c r="C28" t="n">
-        <v>250165.3</v>
+        <v>252237</v>
       </c>
       <c r="D28" t="n">
-        <v>75.5</v>
+        <v>139.3</v>
       </c>
       <c r="E28" t="n">
-        <v>13.3</v>
+        <v>7.2</v>
       </c>
       <c r="F28" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="G28" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="H28" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="I28" t="n">
-        <v>62.5</v>
+        <v>124.9</v>
       </c>
       <c r="J28" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="K28" t="n">
         <v>0.4</v>
@@ -1688,31 +1688,31 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>250165.3</v>
+        <v>252237</v>
       </c>
       <c r="C29" t="n">
-        <v>250165.3</v>
+        <v>252237.1</v>
       </c>
       <c r="D29" t="n">
-        <v>75.40000000000001</v>
+        <v>138.8</v>
       </c>
       <c r="E29" t="n">
-        <v>13.2</v>
+        <v>7.2</v>
       </c>
       <c r="F29" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="G29" t="n">
         <v>1.2</v>
       </c>
       <c r="H29" t="n">
-        <v>7.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I29" t="n">
-        <v>62.2</v>
+        <v>123.3</v>
       </c>
       <c r="J29" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K29" t="n">
         <v>0.4</v>
@@ -1732,43 +1732,43 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>250165.3</v>
+        <v>252237.1</v>
       </c>
       <c r="C30" t="n">
-        <v>250165.4</v>
+        <v>252237.3</v>
       </c>
       <c r="D30" t="n">
-        <v>75</v>
+        <v>136.5</v>
       </c>
       <c r="E30" t="n">
-        <v>13.2</v>
+        <v>7.2</v>
       </c>
       <c r="F30" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G30" t="n">
         <v>0.9</v>
       </c>
       <c r="H30" t="n">
-        <v>7.4</v>
+        <v>8</v>
       </c>
       <c r="I30" t="n">
-        <v>63</v>
+        <v>122.5</v>
       </c>
       <c r="J30" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="K30" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L30" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M30" t="n">
         <v>0.3</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="31">
@@ -1776,31 +1776,31 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>250165.4</v>
+        <v>252237.3</v>
       </c>
       <c r="C31" t="n">
-        <v>250165.5</v>
+        <v>252237.4</v>
       </c>
       <c r="D31" t="n">
-        <v>73.3</v>
+        <v>139</v>
       </c>
       <c r="E31" t="n">
-        <v>13.2</v>
+        <v>7.2</v>
       </c>
       <c r="F31" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G31" t="n">
         <v>1.1</v>
       </c>
-      <c r="G31" t="n">
-        <v>0.8</v>
-      </c>
       <c r="H31" t="n">
-        <v>5.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I31" t="n">
-        <v>62.5</v>
+        <v>123.6</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="K31" t="n">
         <v>0.4</v>
@@ -1809,7 +1809,7 @@
         <v>0.2</v>
       </c>
       <c r="M31" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N31" t="n">
         <v>0.1</v>
@@ -1820,43 +1820,43 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>250165.5</v>
+        <v>252237.4</v>
       </c>
       <c r="C32" t="n">
-        <v>250165.6</v>
+        <v>252237.6</v>
       </c>
       <c r="D32" t="n">
-        <v>72.90000000000001</v>
+        <v>138.8</v>
       </c>
       <c r="E32" t="n">
-        <v>13.2</v>
+        <v>7.2</v>
       </c>
       <c r="F32" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="H32" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
       <c r="I32" t="n">
-        <v>59.4</v>
+        <v>123.7</v>
       </c>
       <c r="J32" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="K32" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L32" t="n">
         <v>0.2</v>
       </c>
       <c r="M32" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N32" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="33">
@@ -1864,31 +1864,31 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>250165.6</v>
+        <v>252237.6</v>
       </c>
       <c r="C33" t="n">
-        <v>250165.6</v>
+        <v>252237.7</v>
       </c>
       <c r="D33" t="n">
-        <v>72.40000000000001</v>
+        <v>138.8</v>
       </c>
       <c r="E33" t="n">
-        <v>13.3</v>
+        <v>7.2</v>
       </c>
       <c r="F33" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>6.3</v>
+        <v>7.8</v>
       </c>
       <c r="I33" t="n">
-        <v>60.6</v>
+        <v>125.2</v>
       </c>
       <c r="J33" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="K33" t="n">
         <v>0.4</v>
@@ -1908,31 +1908,31 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>250165.6</v>
+        <v>252237.7</v>
       </c>
       <c r="C34" t="n">
-        <v>250165.7</v>
+        <v>252237.8</v>
       </c>
       <c r="D34" t="n">
-        <v>74.5</v>
+        <v>139</v>
       </c>
       <c r="E34" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F34" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G34" t="n">
         <v>1.2</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0.9</v>
       </c>
       <c r="H34" t="n">
         <v>8</v>
       </c>
       <c r="I34" t="n">
-        <v>61.6</v>
+        <v>125.1</v>
       </c>
       <c r="J34" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K34" t="n">
         <v>0.4</v>
@@ -1941,7 +1941,7 @@
         <v>0.2</v>
       </c>
       <c r="M34" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N34" t="n">
         <v>0.1</v>
@@ -1952,43 +1952,43 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>250165.7</v>
+        <v>252237.8</v>
       </c>
       <c r="C35" t="n">
-        <v>250165.8</v>
+        <v>252238</v>
       </c>
       <c r="D35" t="n">
-        <v>72.59999999999999</v>
+        <v>137.7</v>
       </c>
       <c r="E35" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F35" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="G35" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="H35" t="n">
-        <v>7.7</v>
+        <v>8.4</v>
       </c>
       <c r="I35" t="n">
-        <v>60.5</v>
+        <v>123.5</v>
       </c>
       <c r="J35" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="K35" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L35" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M35" t="n">
         <v>0.3</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="36">
@@ -1996,43 +1996,43 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>250165.8</v>
+        <v>252238</v>
       </c>
       <c r="C36" t="n">
-        <v>250165.8</v>
+        <v>252238.1</v>
       </c>
       <c r="D36" t="n">
-        <v>72.8</v>
+        <v>138.7</v>
       </c>
       <c r="E36" t="n">
-        <v>13.5</v>
+        <v>7.2</v>
       </c>
       <c r="F36" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G36" t="n">
         <v>1.2</v>
       </c>
       <c r="H36" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="I36" t="n">
-        <v>60.3</v>
+        <v>125.1</v>
       </c>
       <c r="J36" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L36" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M36" t="n">
         <v>0.3</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="37">
@@ -2040,43 +2040,43 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>250165.8</v>
+        <v>252238.1</v>
       </c>
       <c r="C37" t="n">
-        <v>250165.9</v>
+        <v>252238.3</v>
       </c>
       <c r="D37" t="n">
-        <v>76</v>
+        <v>138.5</v>
       </c>
       <c r="E37" t="n">
-        <v>13.6</v>
+        <v>7.2</v>
       </c>
       <c r="F37" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="G37" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="H37" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="I37" t="n">
-        <v>63.7</v>
+        <v>124.8</v>
       </c>
       <c r="J37" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="K37" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L37" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M37" t="n">
         <v>0.3</v>
       </c>
       <c r="N37" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="38">
@@ -2084,31 +2084,31 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>250165.9</v>
+        <v>252238.3</v>
       </c>
       <c r="C38" t="n">
-        <v>250166</v>
+        <v>252238.4</v>
       </c>
       <c r="D38" t="n">
-        <v>71.2</v>
+        <v>139.4</v>
       </c>
       <c r="E38" t="n">
-        <v>13.5</v>
+        <v>7.2</v>
       </c>
       <c r="F38" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="H38" t="n">
-        <v>5.8</v>
+        <v>8.1</v>
       </c>
       <c r="I38" t="n">
-        <v>60.5</v>
+        <v>125.7</v>
       </c>
       <c r="J38" t="n">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="K38" t="n">
         <v>0.4</v>
@@ -2117,7 +2117,7 @@
         <v>0.2</v>
       </c>
       <c r="M38" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N38" t="n">
         <v>0.1</v>
@@ -2128,40 +2128,40 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>250166</v>
+        <v>252238.4</v>
       </c>
       <c r="C39" t="n">
-        <v>250166.1</v>
+        <v>252238.5</v>
       </c>
       <c r="D39" t="n">
-        <v>75.09999999999999</v>
+        <v>138.9</v>
       </c>
       <c r="E39" t="n">
-        <v>13.6</v>
+        <v>7.2</v>
       </c>
       <c r="F39" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="H39" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I39" t="n">
-        <v>61.5</v>
+        <v>123.7</v>
       </c>
       <c r="J39" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="K39" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M39" t="n">
         <v>0.3</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0.5</v>
       </c>
       <c r="N39" t="n">
         <v>0.1</v>
@@ -2172,31 +2172,31 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>250166.1</v>
+        <v>252238.5</v>
       </c>
       <c r="C40" t="n">
-        <v>250166.1</v>
+        <v>252238.7</v>
       </c>
       <c r="D40" t="n">
-        <v>75.90000000000001</v>
+        <v>139.2</v>
       </c>
       <c r="E40" t="n">
-        <v>13.6</v>
+        <v>7.2</v>
       </c>
       <c r="F40" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="G40" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="H40" t="n">
-        <v>6.2</v>
+        <v>7.9</v>
       </c>
       <c r="I40" t="n">
-        <v>63.4</v>
+        <v>125.5</v>
       </c>
       <c r="J40" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="K40" t="n">
         <v>0.4</v>
@@ -2205,10 +2205,10 @@
         <v>0.2</v>
       </c>
       <c r="M40" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="41">
@@ -2216,43 +2216,43 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>250166.1</v>
+        <v>252238.7</v>
       </c>
       <c r="C41" t="n">
-        <v>250166.2</v>
+        <v>252238.8</v>
       </c>
       <c r="D41" t="n">
-        <v>76.59999999999999</v>
+        <v>138.9</v>
       </c>
       <c r="E41" t="n">
-        <v>13.6</v>
+        <v>7.2</v>
       </c>
       <c r="F41" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="H41" t="n">
-        <v>8.6</v>
+        <v>8.1</v>
       </c>
       <c r="I41" t="n">
-        <v>62.7</v>
+        <v>125.1</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="K41" t="n">
         <v>0.4</v>
       </c>
       <c r="L41" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M41" t="n">
         <v>0.4</v>
       </c>
       <c r="N41" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="42">
@@ -2260,43 +2260,43 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>250166.2</v>
+        <v>252238.8</v>
       </c>
       <c r="C42" t="n">
-        <v>250166.3</v>
+        <v>252238.9</v>
       </c>
       <c r="D42" t="n">
-        <v>76.7</v>
+        <v>137.4</v>
       </c>
       <c r="E42" t="n">
-        <v>13.5</v>
+        <v>7.2</v>
       </c>
       <c r="F42" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="G42" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="H42" t="n">
-        <v>7.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I42" t="n">
-        <v>64</v>
+        <v>123</v>
       </c>
       <c r="J42" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="K42" t="n">
         <v>0.4</v>
       </c>
       <c r="L42" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M42" t="n">
         <v>0.4</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="43">
@@ -2304,43 +2304,43 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>250166.3</v>
+        <v>252238.9</v>
       </c>
       <c r="C43" t="n">
-        <v>250166.4</v>
+        <v>252239.1</v>
       </c>
       <c r="D43" t="n">
-        <v>73.8</v>
+        <v>139</v>
       </c>
       <c r="E43" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F43" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="G43" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="H43" t="n">
-        <v>6.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I43" t="n">
-        <v>62.1</v>
+        <v>123.9</v>
       </c>
       <c r="J43" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="K43" t="n">
         <v>0.4</v>
       </c>
       <c r="L43" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="M43" t="n">
         <v>0.4</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44">
@@ -2348,37 +2348,37 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>250166.4</v>
+        <v>252239.1</v>
       </c>
       <c r="C44" t="n">
-        <v>250166.4</v>
+        <v>252239.2</v>
       </c>
       <c r="D44" t="n">
-        <v>74.7</v>
+        <v>138.7</v>
       </c>
       <c r="E44" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F44" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G44" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="H44" t="n">
-        <v>7.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I44" t="n">
-        <v>62.1</v>
+        <v>124.8</v>
       </c>
       <c r="J44" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="K44" t="n">
         <v>0.4</v>
       </c>
       <c r="L44" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M44" t="n">
         <v>0.4</v>
@@ -2392,31 +2392,31 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>250166.4</v>
+        <v>252239.2</v>
       </c>
       <c r="C45" t="n">
-        <v>250166.5</v>
+        <v>252239.4</v>
       </c>
       <c r="D45" t="n">
-        <v>75.2</v>
+        <v>138.6</v>
       </c>
       <c r="E45" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F45" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G45" t="n">
         <v>1.2</v>
       </c>
-      <c r="G45" t="n">
-        <v>0.9</v>
-      </c>
       <c r="H45" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I45" t="n">
-        <v>62.6</v>
+        <v>124.4</v>
       </c>
       <c r="J45" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="K45" t="n">
         <v>0.4</v>
@@ -2428,7 +2428,7 @@
         <v>0.4</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="46">
@@ -2436,43 +2436,43 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>250166.5</v>
+        <v>252239.4</v>
       </c>
       <c r="C46" t="n">
-        <v>250166.6</v>
+        <v>252239.5</v>
       </c>
       <c r="D46" t="n">
-        <v>73.8</v>
+        <v>141.5</v>
       </c>
       <c r="E46" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F46" t="n">
-        <v>1.2</v>
+        <v>2.6</v>
       </c>
       <c r="G46" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="H46" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
       <c r="I46" t="n">
-        <v>61.7</v>
+        <v>125.9</v>
       </c>
       <c r="J46" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="K46" t="n">
         <v>0.4</v>
       </c>
       <c r="L46" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M46" t="n">
         <v>0.4</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="47">
@@ -2480,43 +2480,43 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>250166.6</v>
+        <v>252239.5</v>
       </c>
       <c r="C47" t="n">
-        <v>250166.7</v>
+        <v>252239.6</v>
       </c>
       <c r="D47" t="n">
-        <v>71.8</v>
+        <v>140.3</v>
       </c>
       <c r="E47" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F47" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="G47" t="n">
         <v>0.9</v>
       </c>
       <c r="H47" t="n">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="I47" t="n">
-        <v>59.3</v>
+        <v>126</v>
       </c>
       <c r="J47" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="K47" t="n">
         <v>0.4</v>
       </c>
       <c r="L47" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="M47" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="48">
@@ -2524,43 +2524,43 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>250166.7</v>
+        <v>252239.6</v>
       </c>
       <c r="C48" t="n">
-        <v>250166.7</v>
+        <v>252239.8</v>
       </c>
       <c r="D48" t="n">
-        <v>71.5</v>
+        <v>139.6</v>
       </c>
       <c r="E48" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F48" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G48" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="H48" t="n">
-        <v>6.2</v>
+        <v>8</v>
       </c>
       <c r="I48" t="n">
-        <v>60.8</v>
+        <v>125.8</v>
       </c>
       <c r="J48" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="K48" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L48" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M48" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="49">
@@ -2568,43 +2568,43 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>250166.7</v>
+        <v>252239.8</v>
       </c>
       <c r="C49" t="n">
-        <v>250166.8</v>
+        <v>252239.9</v>
       </c>
       <c r="D49" t="n">
-        <v>74.5</v>
+        <v>137.9</v>
       </c>
       <c r="E49" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F49" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="G49" t="n">
         <v>0.9</v>
       </c>
       <c r="H49" t="n">
-        <v>7.4</v>
+        <v>8</v>
       </c>
       <c r="I49" t="n">
-        <v>62.7</v>
+        <v>124.4</v>
       </c>
       <c r="J49" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="K49" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M49" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="50">
@@ -2612,37 +2612,37 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>250166.8</v>
+        <v>252239.9</v>
       </c>
       <c r="C50" t="n">
-        <v>250166.9</v>
+        <v>252240.1</v>
       </c>
       <c r="D50" t="n">
-        <v>74</v>
+        <v>138.5</v>
       </c>
       <c r="E50" t="n">
-        <v>13.4</v>
+        <v>7.2</v>
       </c>
       <c r="F50" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="G50" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="H50" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
       <c r="I50" t="n">
-        <v>61.8</v>
+        <v>124.9</v>
       </c>
       <c r="J50" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="K50" t="n">
         <v>0.4</v>
       </c>
       <c r="L50" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="M50" t="n">
         <v>0.4</v>
@@ -2656,43 +2656,43 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>250166.9</v>
+        <v>252240.1</v>
       </c>
       <c r="C51" t="n">
-        <v>250167</v>
+        <v>252240.2</v>
       </c>
       <c r="D51" t="n">
-        <v>72.5</v>
+        <v>142.7</v>
       </c>
       <c r="E51" t="n">
-        <v>13.5</v>
+        <v>7.2</v>
       </c>
       <c r="F51" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G51" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="H51" t="n">
-        <v>7.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I51" t="n">
-        <v>60.5</v>
+        <v>128.4</v>
       </c>
       <c r="J51" t="n">
-        <v>1.3</v>
+        <v>2.2</v>
       </c>
       <c r="K51" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L51" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="M51" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="52">
@@ -2700,43 +2700,219 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>250167</v>
+        <v>252240.2</v>
       </c>
       <c r="C52" t="n">
-        <v>250167</v>
+        <v>252240.3</v>
       </c>
       <c r="D52" t="n">
-        <v>78.8</v>
+        <v>142.8</v>
       </c>
       <c r="E52" t="n">
-        <v>13.5</v>
+        <v>7.2</v>
       </c>
       <c r="F52" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="G52" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="I52" t="n">
+        <v>128.3</v>
+      </c>
+      <c r="J52" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="n">
+        <v>252240.3</v>
+      </c>
+      <c r="C53" t="n">
+        <v>252240.5</v>
+      </c>
+      <c r="D53" t="n">
+        <v>141.4</v>
+      </c>
+      <c r="E53" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G53" t="n">
         <v>1</v>
       </c>
-      <c r="H52" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="I52" t="n">
-        <v>63.9</v>
-      </c>
-      <c r="J52" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="K52" t="n">
+      <c r="H53" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="I53" t="n">
+        <v>126.6</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K53" t="n">
         <v>0.5</v>
       </c>
-      <c r="L52" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M52" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="N52" t="n">
-        <v>0.1</v>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="n">
+        <v>252240.5</v>
+      </c>
+      <c r="C54" t="n">
+        <v>252240.6</v>
+      </c>
+      <c r="D54" t="n">
+        <v>145.2</v>
+      </c>
+      <c r="E54" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H54" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="I54" t="n">
+        <v>129.1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="n">
+        <v>252240.6</v>
+      </c>
+      <c r="C55" t="n">
+        <v>252240.8</v>
+      </c>
+      <c r="D55" t="n">
+        <v>141.1</v>
+      </c>
+      <c r="E55" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H55" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="I55" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="J55" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="n">
+        <v>252240.8</v>
+      </c>
+      <c r="C56" t="n">
+        <v>252240.9</v>
+      </c>
+      <c r="D56" t="n">
+        <v>139.8</v>
+      </c>
+      <c r="E56" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H56" t="n">
+        <v>8</v>
+      </c>
+      <c r="I56" t="n">
+        <v>125.9</v>
+      </c>
+      <c r="J56" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>